<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-08-30
</commit_message>
<xml_diff>
--- a/HK_Swing_Pattern.xlsx
+++ b/HK_Swing_Pattern.xlsx
@@ -27170,9 +27170,7 @@
       </c>
       <c r="O426" s="2" t="inlineStr"/>
       <c r="P426" s="2" t="inlineStr"/>
-      <c r="Q426" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q426" s="2" t="inlineStr"/>
       <c r="R426" s="2" t="n">
         <v>-1</v>
       </c>
@@ -33286,7 +33284,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=1.8x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300/HK恒指HSI.HI(jianxin)/美股S&amp;P500; 基准缺失时跳过此门)</t>
+          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=1.8x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
         </is>
       </c>
     </row>

</xml_diff>